<commit_message>
Fix corrupcion Excel: populado por cadena (preserva namespaces mc/xr2/xr3)
CAUSA: la plantilla congelada se habia limpiado con ElementTree, que renombraba
los namespaces del worksheet a ns1/ns2/ns3 y dejaba mc:Ignorable="x14ac xr xr2 xr3"
apuntando a prefijos ya inexistentes -> Excel "reparaba" el fichero al abrirlo.

- Plantilla re-congelada limpiando celdas por manipulacion de CADENA (sin reparsear):
  namespaces mc/x14ac/xr/xr2/xr3 + mc:Ignorable intactos byte a byte, 10.500 formulas
  y 2 graficos conservados, abre en Informe Subasta.
- populate-xlsx.ts reescrito: StringSheet (regex) en vez de DOMParser+XMLSerializer,
  que podia soltar xmlns:xr2/xr3 (declarados pero solo citados en mc:Ignorable) y
  recorromper. Inserta celdas nuevas en fincas 2+ conservando sus formulas. Verificado
  en Python contra la plantilla real: namespaces intactos, valores y fincas correctos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla/Calculo_Deuda_y_Subasta.xlsx
+++ b/public/plantilla/Calculo_Deuda_y_Subasta.xlsx
@@ -3647,13 +3647,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AE60"/>
-  <sheetFormatPr defaultRowHeight="14.5" ns3:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="3" width="10" customWidth="1"/>
@@ -3682,7 +3682,7 @@
     <col min="31" max="31" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="26.15" customHeight="1" ns3:dyDescent="0.35">
+    <row r="1" spans="1:31" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="176" t="s">
         <v>41</v>
       </c>
@@ -3717,7 +3717,7 @@
       <c r="AD1" s="138"/>
       <c r="AE1" s="138"/>
     </row>
-    <row r="2" spans="1:31" ns3:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" s="169" t="s">
         <v>42</v>
       </c>
@@ -3752,7 +3752,7 @@
       <c r="AD2" s="138"/>
       <c r="AE2" s="138"/>
     </row>
-    <row r="4" spans="1:31" ht="19" customHeight="1" ns3:dyDescent="0.35">
+    <row r="4" spans="1:31" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="152" t="s">
         <v>43</v>
       </c>
@@ -3787,7 +3787,7 @@
       <c r="AD4" s="147"/>
       <c r="AE4" s="148"/>
     </row>
-    <row r="5" spans="1:31" ns3:dyDescent="0.35">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" s="159" t="s">
         <v>44</v>
       </c>
@@ -3832,7 +3832,7 @@
       <c r="AD5" s="147"/>
       <c r="AE5" s="148"/>
     </row>
-    <row r="6" spans="1:31" ht="22" customHeight="1" ns3:dyDescent="0.35">
+    <row r="6" spans="1:31" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="177">
         <f>$K$13</f>
         <v>0</v>
@@ -3883,7 +3883,7 @@
       <c r="AD6" s="154"/>
       <c r="AE6" s="155"/>
     </row>
-    <row r="7" spans="1:31" ht="14.15" customHeight="1" ns3:dyDescent="0.35">
+    <row r="7" spans="1:31" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="156"/>
       <c r="B7" s="157"/>
       <c r="C7" s="157"/>
@@ -3916,7 +3916,7 @@
       <c r="AD7" s="157"/>
       <c r="AE7" s="158"/>
     </row>
-    <row r="8" spans="1:31" ns3:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" s="74" t="s">
         <v>50</v>
       </c>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="Y8" s="116"/>
     </row>
-    <row r="9" spans="1:31" ht="19" customHeight="1" ns3:dyDescent="0.35">
+    <row r="9" spans="1:31" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="152" t="s">
         <v>55</v>
       </c>
@@ -3966,7 +3966,7 @@
       <c r="Z9" s="147"/>
       <c r="AA9" s="148"/>
     </row>
-    <row r="10" spans="1:31" ns3:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" s="146" t="s">
         <v>57</v>
       </c>
@@ -4005,7 +4005,7 @@
       <c r="Z10" s="147"/>
       <c r="AA10" s="148"/>
     </row>
-    <row r="11" spans="1:31" ns3:dyDescent="0.35">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" s="146" t="s">
         <v>62</v>
       </c>
@@ -4045,7 +4045,7 @@
       <c r="Z11" s="147"/>
       <c r="AA11" s="148"/>
     </row>
-    <row r="12" spans="1:31" ns3:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" s="146" t="s">
         <v>66</v>
       </c>
@@ -4081,7 +4081,7 @@
       <c r="Z12" s="154"/>
       <c r="AA12" s="155"/>
     </row>
-    <row r="13" spans="1:31" ns3:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" s="146" t="s">
         <v>70</v>
       </c>
@@ -4112,7 +4112,7 @@
       <c r="Z13" s="157"/>
       <c r="AA13" s="158"/>
     </row>
-    <row r="14" spans="1:31" ns3:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" s="146" t="s">
         <v>72</v>
       </c>
@@ -4130,7 +4130,7 @@
       <c r="L14" s="147"/>
       <c r="M14" s="148"/>
     </row>
-    <row r="15" spans="1:31" ht="19" customHeight="1" ns3:dyDescent="0.35">
+    <row r="15" spans="1:31" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="146" t="s">
         <v>74</v>
       </c>
@@ -4163,7 +4163,7 @@
       <c r="Z15" s="147"/>
       <c r="AA15" s="148"/>
     </row>
-    <row r="16" spans="1:31" ns3:dyDescent="0.35">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" s="146" t="s">
         <v>77</v>
       </c>
@@ -4206,7 +4206,7 @@
       <c r="Z16" s="147"/>
       <c r="AA16" s="148"/>
     </row>
-    <row r="17" spans="1:31" ns3:dyDescent="0.35">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" s="146" t="s">
         <v>81</v>
       </c>
@@ -4252,7 +4252,7 @@
       <c r="Z17" s="147"/>
       <c r="AA17" s="148"/>
     </row>
-    <row r="19" spans="1:31" ht="19" customHeight="1" ns3:dyDescent="0.35">
+    <row r="19" spans="1:31" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="152" t="s">
         <v>85</v>
       </c>
@@ -4284,7 +4284,7 @@
       <c r="Z19" s="147"/>
       <c r="AA19" s="148"/>
     </row>
-    <row r="20" spans="1:31" ht="15.75" customHeight="1" ns3:dyDescent="0.35">
+    <row r="20" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="146" t="s">
         <v>87</v>
       </c>
@@ -4323,7 +4323,7 @@
       <c r="Z20" s="147"/>
       <c r="AA20" s="148"/>
     </row>
-    <row r="21" spans="1:31" ht="15.75" customHeight="1" ns3:dyDescent="0.35">
+    <row r="21" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="146" t="s">
         <v>92</v>
       </c>
@@ -4360,7 +4360,7 @@
       <c r="Z21" s="147"/>
       <c r="AA21" s="148"/>
     </row>
-    <row r="22" spans="1:31" ht="15.75" customHeight="1" ns3:dyDescent="0.35">
+    <row r="22" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="146" t="s">
         <v>96</v>
       </c>
@@ -4397,7 +4397,7 @@
       <c r="Z22" s="147"/>
       <c r="AA22" s="148"/>
     </row>
-    <row r="23" spans="1:31" ht="15.75" customHeight="1" ns3:dyDescent="0.35">
+    <row r="23" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="146" t="s">
         <v>99</v>
       </c>
@@ -4434,7 +4434,7 @@
       <c r="Z23" s="147"/>
       <c r="AA23" s="148"/>
     </row>
-    <row r="24" spans="1:31" ht="15.75" customHeight="1" ns3:dyDescent="0.35">
+    <row r="24" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="146" t="s">
         <v>102</v>
       </c>
@@ -4473,7 +4473,7 @@
       <c r="Z24" s="147"/>
       <c r="AA24" s="148"/>
     </row>
-    <row r="25" spans="1:31" ht="15.75" customHeight="1" ns3:dyDescent="0.35">
+    <row r="25" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="O25" s="146" t="s">
         <v>106</v>
       </c>
@@ -4492,7 +4492,7 @@
       <c r="Z25" s="147"/>
       <c r="AA25" s="148"/>
     </row>
-    <row r="27" spans="1:31" ht="19" customHeight="1" ns3:dyDescent="0.35">
+    <row r="27" spans="1:31" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="152" t="s">
         <v>107</v>
       </c>
@@ -4527,7 +4527,7 @@
       <c r="AD27" s="147"/>
       <c r="AE27" s="148"/>
     </row>
-    <row r="28" spans="1:31" ht="15" customHeight="1" ns3:dyDescent="0.35">
+    <row r="28" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="151" t="s">
         <v>108</v>
       </c>
@@ -4578,7 +4578,7 @@
       <c r="AD28" s="147"/>
       <c r="AE28" s="148"/>
     </row>
-    <row r="29" spans="1:31" ht="34" customHeight="1" ns3:dyDescent="0.35">
+    <row r="29" spans="1:31" ht="34" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>117</v>
       </c>
@@ -4673,7 +4673,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="30" spans="1:31" ns3:dyDescent="0.35">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -4757,7 +4757,7 @@
       <c r="AD30" s="5"/>
       <c r="AE30" s="5"/>
     </row>
-    <row r="31" spans="1:31" ns3:dyDescent="0.35">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -4841,7 +4841,7 @@
       <c r="AD31" s="5"/>
       <c r="AE31" s="5"/>
     </row>
-    <row r="32" spans="1:31" ns3:dyDescent="0.35">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4925,7 +4925,7 @@
       <c r="AD32" s="5"/>
       <c r="AE32" s="5"/>
     </row>
-    <row r="33" spans="1:31" ns3:dyDescent="0.35">
+    <row r="33" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -5009,7 +5009,7 @@
       <c r="AD33" s="5"/>
       <c r="AE33" s="5"/>
     </row>
-    <row r="34" spans="1:31" ns3:dyDescent="0.35">
+    <row r="34" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A34" s="5"/>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -5093,7 +5093,7 @@
       <c r="AD34" s="5"/>
       <c r="AE34" s="5"/>
     </row>
-    <row r="35" spans="1:31" ns3:dyDescent="0.35">
+    <row r="35" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -5177,7 +5177,7 @@
       <c r="AD35" s="5"/>
       <c r="AE35" s="5"/>
     </row>
-    <row r="36" spans="1:31" ns3:dyDescent="0.35">
+    <row r="36" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -5261,7 +5261,7 @@
       <c r="AD36" s="5"/>
       <c r="AE36" s="5"/>
     </row>
-    <row r="37" spans="1:31" ns3:dyDescent="0.35">
+    <row r="37" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A37" s="5"/>
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
@@ -5345,7 +5345,7 @@
       <c r="AD37" s="5"/>
       <c r="AE37" s="5"/>
     </row>
-    <row r="38" spans="1:31" ns3:dyDescent="0.35">
+    <row r="38" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
@@ -5429,7 +5429,7 @@
       <c r="AD38" s="5"/>
       <c r="AE38" s="5"/>
     </row>
-    <row r="39" spans="1:31" ns3:dyDescent="0.35">
+    <row r="39" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A39" s="5"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -5513,7 +5513,7 @@
       <c r="AD39" s="5"/>
       <c r="AE39" s="5"/>
     </row>
-    <row r="40" spans="1:31" ns3:dyDescent="0.35">
+    <row r="40" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A40" s="5"/>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
@@ -5597,7 +5597,7 @@
       <c r="AD40" s="5"/>
       <c r="AE40" s="5"/>
     </row>
-    <row r="41" spans="1:31" ns3:dyDescent="0.35">
+    <row r="41" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A41" s="5"/>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
@@ -5681,7 +5681,7 @@
       <c r="AD41" s="5"/>
       <c r="AE41" s="5"/>
     </row>
-    <row r="42" spans="1:31" ns3:dyDescent="0.35">
+    <row r="42" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A42" s="5"/>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
@@ -5765,7 +5765,7 @@
       <c r="AD42" s="5"/>
       <c r="AE42" s="5"/>
     </row>
-    <row r="43" spans="1:31" ns3:dyDescent="0.35">
+    <row r="43" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A43" s="5"/>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -5849,7 +5849,7 @@
       <c r="AD43" s="5"/>
       <c r="AE43" s="5"/>
     </row>
-    <row r="44" spans="1:31" ns3:dyDescent="0.35">
+    <row r="44" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A44" s="5"/>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
@@ -5933,7 +5933,7 @@
       <c r="AD44" s="5"/>
       <c r="AE44" s="5"/>
     </row>
-    <row r="45" spans="1:31" ns3:dyDescent="0.35">
+    <row r="45" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A45" s="5"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
@@ -6017,7 +6017,7 @@
       <c r="AD45" s="5"/>
       <c r="AE45" s="5"/>
     </row>
-    <row r="46" spans="1:31" ns3:dyDescent="0.35">
+    <row r="46" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A46" s="5"/>
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
@@ -6101,7 +6101,7 @@
       <c r="AD46" s="5"/>
       <c r="AE46" s="5"/>
     </row>
-    <row r="47" spans="1:31" ns3:dyDescent="0.35">
+    <row r="47" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A47" s="5"/>
       <c r="B47" s="5"/>
       <c r="C47" s="5"/>
@@ -6185,7 +6185,7 @@
       <c r="AD47" s="5"/>
       <c r="AE47" s="5"/>
     </row>
-    <row r="48" spans="1:31" ns3:dyDescent="0.35">
+    <row r="48" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A48" s="5"/>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
@@ -6269,7 +6269,7 @@
       <c r="AD48" s="5"/>
       <c r="AE48" s="5"/>
     </row>
-    <row r="49" spans="1:31" ns3:dyDescent="0.35">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A49" s="5"/>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
@@ -6353,7 +6353,7 @@
       <c r="AD49" s="5"/>
       <c r="AE49" s="5"/>
     </row>
-    <row r="50" spans="1:31" ns3:dyDescent="0.35">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A50" s="5"/>
       <c r="B50" s="5"/>
       <c r="C50" s="5"/>
@@ -6437,7 +6437,7 @@
       <c r="AD50" s="5"/>
       <c r="AE50" s="5"/>
     </row>
-    <row r="51" spans="1:31" ns3:dyDescent="0.35">
+    <row r="51" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A51" s="5"/>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
@@ -6521,7 +6521,7 @@
       <c r="AD51" s="5"/>
       <c r="AE51" s="5"/>
     </row>
-    <row r="52" spans="1:31" ns3:dyDescent="0.35">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A52" s="5"/>
       <c r="B52" s="5"/>
       <c r="C52" s="5"/>
@@ -6605,7 +6605,7 @@
       <c r="AD52" s="5"/>
       <c r="AE52" s="5"/>
     </row>
-    <row r="53" spans="1:31" ns3:dyDescent="0.35">
+    <row r="53" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A53" s="5"/>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
@@ -6689,7 +6689,7 @@
       <c r="AD53" s="5"/>
       <c r="AE53" s="5"/>
     </row>
-    <row r="54" spans="1:31" ns3:dyDescent="0.35">
+    <row r="54" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A54" s="5"/>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
@@ -6773,7 +6773,7 @@
       <c r="AD54" s="5"/>
       <c r="AE54" s="5"/>
     </row>
-    <row r="55" spans="1:31" ns3:dyDescent="0.35">
+    <row r="55" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A55" s="5"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
@@ -6857,7 +6857,7 @@
       <c r="AD55" s="5"/>
       <c r="AE55" s="5"/>
     </row>
-    <row r="56" spans="1:31" ns3:dyDescent="0.35">
+    <row r="56" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A56" s="5"/>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
@@ -6941,7 +6941,7 @@
       <c r="AD56" s="5"/>
       <c r="AE56" s="5"/>
     </row>
-    <row r="57" spans="1:31" ns3:dyDescent="0.35">
+    <row r="57" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A57" s="5"/>
       <c r="B57" s="5"/>
       <c r="C57" s="5"/>
@@ -7025,7 +7025,7 @@
       <c r="AD57" s="5"/>
       <c r="AE57" s="5"/>
     </row>
-    <row r="58" spans="1:31" ns3:dyDescent="0.35">
+    <row r="58" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A58" s="5"/>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
@@ -7109,7 +7109,7 @@
       <c r="AD58" s="5"/>
       <c r="AE58" s="5"/>
     </row>
-    <row r="59" spans="1:31" ns3:dyDescent="0.35">
+    <row r="59" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A59" s="5"/>
       <c r="B59" s="5"/>
       <c r="C59" s="5"/>
@@ -7193,7 +7193,7 @@
       <c r="AD59" s="5"/>
       <c r="AE59" s="5"/>
     </row>
-    <row r="60" spans="1:31" ns3:dyDescent="0.35">
+    <row r="60" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
         <v>37</v>
       </c>
@@ -7402,16 +7402,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="D20" ns2:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D20" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"FIJO,VARIABLE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B30:B59 D21 R10" ns2:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B30:B59 D21 R10" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D24" ns2:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D24" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="Y20:Y25" ns2:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" sqref="Y20:Y25" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"✓,✗"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>